<commit_message>
Log v1.3 design redesign in changelog
</commit_message>
<xml_diff>
--- a/tripplanner_changelog.xlsx
+++ b/tripplanner_changelog.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gogle\Claude\Projects\TripPlanner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C42D1848-0132-426B-B2A2-8E165EAB201F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADA6F8F0-0C03-403B-ABDC-817B4D209233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="13995" yWindow="2490" windowWidth="23760" windowHeight="17655" xr2:uid="{86CE85FA-8EFB-405C-82A3-7763046D7446}"/>
+    <workbookView xWindow="465" yWindow="1650" windowWidth="23760" windowHeight="17655" xr2:uid="{86CE85FA-8EFB-405C-82A3-7763046D7446}"/>
   </bookViews>
   <sheets>
     <sheet name="変更履歴" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="52">
   <si>
     <t>バージョン</t>
   </si>
@@ -180,6 +180,21 @@
   </si>
   <si>
     <t>車の区間は実道路に沿ったルート線＋距離・所要時間をポップアップ表示するよう変更。電車の区間は線路風の白い破線を重ねて表示するよう変更</t>
+  </si>
+  <si>
+    <t>v1.3</t>
+  </si>
+  <si>
+    <t>2026/07/13</t>
+  </si>
+  <si>
+    <t>背景・カード・ボタン・フォントを暖色系（クリーム×テラコッタ）パレットとZen Maru Gothicフォントに刷新</t>
+  </si>
+  <si>
+    <t>デザイン変更</t>
+  </si>
+  <si>
+    <t>ヘッダー・カード・day-tabs・予定行・タグ・モーダル・地図の配色を暖色系パレットに統一。移動手段の地図ルート色もパレットに合わせて調整。HTML構造/JSロジックは変更なし</t>
   </si>
 </sst>
 </file>
@@ -590,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62BC3060-54A5-4605-B70E-1E9C84D367F5}">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -941,6 +956,46 @@
         <v>40</v>
       </c>
     </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Log v1.4 Gemini AI integration in changelog
</commit_message>
<xml_diff>
--- a/tripplanner_changelog.xlsx
+++ b/tripplanner_changelog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gogle\Claude\Projects\TripPlanner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADA6F8F0-0C03-403B-ABDC-817B4D209233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B087F1D2-8978-429F-8FD6-0B2555002487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="465" yWindow="1650" windowWidth="23760" windowHeight="17655" xr2:uid="{86CE85FA-8EFB-405C-82A3-7763046D7446}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="63">
   <si>
     <t>バージョン</t>
   </si>
@@ -195,6 +195,39 @@
   </si>
   <si>
     <t>ヘッダー・カード・day-tabs・予定行・タグ・モーダル・地図の配色を暖色系パレットに統一。移動手段の地図ルート色もパレットに合わせて調整。HTML構造/JSロジックは変更なし</t>
+  </si>
+  <si>
+    <t>v1.4</t>
+  </si>
+  <si>
+    <t>2026/07/14</t>
+  </si>
+  <si>
+    <t>Gemini API連携を新規追加。_nominatim_search()共通化、_call_gemini()+TRIP_SCHEMAで構造化JSON生成、POST /api/ai/suggest（文章から旅程自動生成）、POST /api/ai/import（xlsx/画像/PDFのしおりを取り込み）を追加</t>
+  </si>
+  <si>
+    <t>AI連携</t>
+  </si>
+  <si>
+    <t>「+ 新しい旅行」に手動/AI提案/ファイル取り込みの3択モーダルを追加。AI提案・取り込みモーダルとnormalizeAiTrip()を新設</t>
+  </si>
+  <si>
+    <t>app/requirements.txt / .env.example / DEPLOY.md</t>
+  </si>
+  <si>
+    <t>openpyxl・python-multipartを追加、GEMINI_API_KEY環境変数とGoogle AI Studioでのキー取得手順を追加</t>
+  </si>
+  <si>
+    <t>不具合修正: gemini-2.5-flashが新規アカウントで利用不可だったためgemini-3-flash-previewに変更</t>
+  </si>
+  <si>
+    <t>不具合修正</t>
+  </si>
+  <si>
+    <t>不具合修正: AIが生成する場所名が詳細住所すぎてNominatimでジオコーディングできず地図にピンが立たなかった問題を、プロンプト調整（施設名・地名のみを返すよう指示）で修正</t>
+  </si>
+  <si>
+    <t>AI連携・地図</t>
   </si>
 </sst>
 </file>
@@ -605,7 +638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62BC3060-54A5-4605-B70E-1E9C84D367F5}">
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -996,6 +1029,106 @@
         <v>17</v>
       </c>
     </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Log geocoding country-restriction fix in changelog
</commit_message>
<xml_diff>
--- a/tripplanner_changelog.xlsx
+++ b/tripplanner_changelog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gogle\Claude\Projects\TripPlanner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B087F1D2-8978-429F-8FD6-0B2555002487}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{497BBDCB-9561-4D64-A99B-96254FD094D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="465" yWindow="1650" windowWidth="23760" windowHeight="17655" xr2:uid="{86CE85FA-8EFB-405C-82A3-7763046D7446}"/>
   </bookViews>
@@ -638,7 +638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62BC3060-54A5-4605-B70E-1E9C84D367F5}">
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:CA30"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -969,7 +969,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:79">
       <c r="A17" s="2" t="s">
         <v>44</v>
       </c>
@@ -989,7 +989,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:79">
       <c r="A18" s="2" t="s">
         <v>47</v>
       </c>
@@ -1009,7 +1009,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:79">
       <c r="A19" s="2" t="s">
         <v>47</v>
       </c>
@@ -1029,7 +1029,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:79">
       <c r="A20" s="2" t="s">
         <v>52</v>
       </c>
@@ -1049,7 +1049,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:79">
       <c r="A21" s="2" t="s">
         <v>52</v>
       </c>
@@ -1069,7 +1069,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:79">
       <c r="A22" s="2" t="s">
         <v>52</v>
       </c>
@@ -1089,7 +1089,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:79">
       <c r="A23" s="2" t="s">
         <v>52</v>
       </c>
@@ -1109,7 +1109,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:79">
       <c r="A24" s="2" t="s">
         <v>52</v>
       </c>
@@ -1127,6 +1127,366 @@
       </c>
       <c r="F24" s="2" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="25" spans="1:79">
+      <c r="A25" s="2">
+        <v>118</v>
+      </c>
+      <c r="B25" s="2">
+        <v>49</v>
+      </c>
+      <c r="C25" s="2">
+        <v>46</v>
+      </c>
+      <c r="D25" s="2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:79">
+      <c r="A26" s="2">
+        <v>97</v>
+      </c>
+      <c r="B26" s="2">
+        <v>112</v>
+      </c>
+      <c r="C26" s="2">
+        <v>112</v>
+      </c>
+      <c r="D26" s="2">
+        <v>47</v>
+      </c>
+      <c r="E26" s="2">
+        <v>109</v>
+      </c>
+      <c r="F26" s="2">
+        <v>97</v>
+      </c>
+      <c r="G26" s="2">
+        <v>105</v>
+      </c>
+      <c r="H26" s="2">
+        <v>110</v>
+      </c>
+      <c r="I26" s="2">
+        <v>46</v>
+      </c>
+      <c r="J26" s="2">
+        <v>112</v>
+      </c>
+      <c r="K26" s="2">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="27" spans="1:79">
+      <c r="A27" s="2">
+        <v>50</v>
+      </c>
+      <c r="B27" s="2">
+        <v>48</v>
+      </c>
+      <c r="C27" s="2">
+        <v>50</v>
+      </c>
+      <c r="D27" s="2">
+        <v>54</v>
+      </c>
+      <c r="E27" s="2">
+        <v>47</v>
+      </c>
+      <c r="F27" s="2">
+        <v>48</v>
+      </c>
+      <c r="G27" s="2">
+        <v>55</v>
+      </c>
+      <c r="H27" s="2">
+        <v>47</v>
+      </c>
+      <c r="I27" s="2">
+        <v>49</v>
+      </c>
+      <c r="J27" s="2">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="28" spans="1:79">
+      <c r="A28" s="2">
+        <v>19981</v>
+      </c>
+      <c r="B28" s="2">
+        <v>20855</v>
+      </c>
+      <c r="C28" s="2">
+        <v>21512</v>
+      </c>
+      <c r="D28" s="2">
+        <v>20462</v>
+      </c>
+      <c r="E28" s="2">
+        <v>27491</v>
+      </c>
+      <c r="F28" s="2">
+        <v>58</v>
+      </c>
+      <c r="G28" s="2">
+        <v>32</v>
+      </c>
+      <c r="H28" s="2">
+        <v>78</v>
+      </c>
+      <c r="I28" s="2">
+        <v>111</v>
+      </c>
+      <c r="J28" s="2">
+        <v>109</v>
+      </c>
+      <c r="K28" s="2">
+        <v>105</v>
+      </c>
+      <c r="L28" s="2">
+        <v>110</v>
+      </c>
+      <c r="M28" s="2">
+        <v>97</v>
+      </c>
+      <c r="N28" s="2">
+        <v>116</v>
+      </c>
+      <c r="O28" s="2">
+        <v>105</v>
+      </c>
+      <c r="P28" s="2">
+        <v>109</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>12364</v>
+      </c>
+      <c r="R28" s="2">
+        <v>21516</v>
+      </c>
+      <c r="S28" s="2">
+        <v>21517</v>
+      </c>
+      <c r="T28" s="2">
+        <v>26045</v>
+      </c>
+      <c r="U28" s="2">
+        <v>35373</v>
+      </c>
+      <c r="V28" s="2">
+        <v>12434</v>
+      </c>
+      <c r="W28" s="2">
+        <v>28023</v>
+      </c>
+      <c r="X28" s="2">
+        <v>22806</v>
+      </c>
+      <c r="Y28" s="2">
+        <v>12539</v>
+      </c>
+      <c r="Z28" s="2">
+        <v>21029</v>
+      </c>
+      <c r="AA28" s="2">
+        <v>30476</v>
+      </c>
+      <c r="AB28" s="2">
+        <v>12398</v>
+      </c>
+      <c r="AC28" s="2">
+        <v>35492</v>
+      </c>
+      <c r="AD28" s="2">
+        <v>12387</v>
+      </c>
+      <c r="AE28" s="2">
+        <v>12383</v>
+      </c>
+      <c r="AF28" s="2">
+        <v>22580</v>
+      </c>
+      <c r="AG28" s="2">
+        <v>25152</v>
+      </c>
+      <c r="AH28" s="2">
+        <v>12395</v>
+      </c>
+      <c r="AI28" s="2">
+        <v>12472</v>
+      </c>
+      <c r="AJ28" s="2">
+        <v>12458</v>
+      </c>
+      <c r="AK28" s="2">
+        <v>12467</v>
+      </c>
+      <c r="AL28" s="2">
+        <v>12540</v>
+      </c>
+      <c r="AM28" s="2">
+        <v>12487</v>
+      </c>
+      <c r="AN28" s="2">
+        <v>12451</v>
+      </c>
+      <c r="AO28" s="2">
+        <v>12531</v>
+      </c>
+      <c r="AP28" s="2">
+        <v>12464</v>
+      </c>
+      <c r="AQ28" s="2">
+        <v>12377</v>
+      </c>
+      <c r="AR28" s="2">
+        <v>12427</v>
+      </c>
+      <c r="AS28" s="2">
+        <v>12371</v>
+      </c>
+      <c r="AT28" s="2">
+        <v>12392</v>
+      </c>
+      <c r="AU28" s="2">
+        <v>12364</v>
+      </c>
+      <c r="AV28" s="2">
+        <v>12354</v>
+      </c>
+      <c r="AW28" s="2">
+        <v>12387</v>
+      </c>
+      <c r="AX28" s="2">
+        <v>12383</v>
+      </c>
+      <c r="AY28" s="2">
+        <v>12383</v>
+      </c>
+      <c r="AZ28" s="2">
+        <v>12417</v>
+      </c>
+      <c r="BA28" s="2">
+        <v>12289</v>
+      </c>
+      <c r="BB28" s="2">
+        <v>99</v>
+      </c>
+      <c r="BC28" s="2">
+        <v>111</v>
+      </c>
+      <c r="BD28" s="2">
+        <v>117</v>
+      </c>
+      <c r="BE28" s="2">
+        <v>110</v>
+      </c>
+      <c r="BF28" s="2">
+        <v>116</v>
+      </c>
+      <c r="BG28" s="2">
+        <v>114</v>
+      </c>
+      <c r="BH28" s="2">
+        <v>121</v>
+      </c>
+      <c r="BI28" s="2">
+        <v>99</v>
+      </c>
+      <c r="BJ28" s="2">
+        <v>111</v>
+      </c>
+      <c r="BK28" s="2">
+        <v>100</v>
+      </c>
+      <c r="BL28" s="2">
+        <v>101</v>
+      </c>
+      <c r="BM28" s="2">
+        <v>115</v>
+      </c>
+      <c r="BN28" s="2">
+        <v>61</v>
+      </c>
+      <c r="BO28" s="2">
+        <v>106</v>
+      </c>
+      <c r="BP28" s="2">
+        <v>112</v>
+      </c>
+      <c r="BQ28" s="2">
+        <v>12391</v>
+      </c>
+      <c r="BR28" s="2">
+        <v>26908</v>
+      </c>
+      <c r="BS28" s="2">
+        <v>32034</v>
+      </c>
+      <c r="BT28" s="2">
+        <v>12434</v>
+      </c>
+      <c r="BU28" s="2">
+        <v>26085</v>
+      </c>
+      <c r="BV28" s="2">
+        <v>26412</v>
+      </c>
+      <c r="BW28" s="2">
+        <v>22269</v>
+      </c>
+      <c r="BX28" s="2">
+        <v>20869</v>
+      </c>
+      <c r="BY28" s="2">
+        <v>12395</v>
+      </c>
+      <c r="BZ28" s="2">
+        <v>38480</v>
+      </c>
+      <c r="CA28" s="2">
+        <v>23450</v>
+      </c>
+    </row>
+    <row r="29" spans="1:79">
+      <c r="A29" s="2">
+        <v>19981</v>
+      </c>
+      <c r="B29" s="2">
+        <v>20855</v>
+      </c>
+      <c r="C29" s="2">
+        <v>21512</v>
+      </c>
+      <c r="D29" s="2">
+        <v>20462</v>
+      </c>
+      <c r="E29" s="2">
+        <v>27491</v>
+      </c>
+    </row>
+    <row r="30" spans="1:79">
+      <c r="A30" s="2">
+        <v>65</v>
+      </c>
+      <c r="B30" s="2">
+        <v>73</v>
+      </c>
+      <c r="C30" s="2">
+        <v>36899</v>
+      </c>
+      <c r="D30" s="2">
+        <v>25658</v>
+      </c>
+      <c r="E30" s="2">
+        <v>12539</v>
+      </c>
+      <c r="F30" s="2">
+        <v>22320</v>
+      </c>
+      <c r="G30" s="2">
+        <v>22259</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Log v1.5 layout redesign and waypoint routing in changelog
</commit_message>
<xml_diff>
--- a/tripplanner_changelog.xlsx
+++ b/tripplanner_changelog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gogle\Claude\Projects\TripPlanner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{497BBDCB-9561-4D64-A99B-96254FD094D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D91779FD-A234-4A6A-8AEF-4A7C9BA28FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="465" yWindow="1650" windowWidth="23760" windowHeight="17655" xr2:uid="{86CE85FA-8EFB-405C-82A3-7763046D7446}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="70">
   <si>
     <t>バージョン</t>
   </si>
@@ -228,6 +228,27 @@
   </si>
   <si>
     <t>AI連携・地図</t>
+  </si>
+  <si>
+    <t>v1.5</t>
+  </si>
+  <si>
+    <t>旅行選択をプルダウンから左サイドバー（年度ごとにグループ化、日付+プラン名表示）に変更</t>
+  </si>
+  <si>
+    <t>旅程カード内に選択中の日付バッジを表示し、日タブもカード内に移動</t>
+  </si>
+  <si>
+    <t>プラン名を大きな見出しとして表示し、鉛筆アイコンからその場で編集できるように変更</t>
+  </si>
+  <si>
+    <t>「予定を追加」「日を追加」ボタンを旅程カードの上部に移動</t>
+  </si>
+  <si>
+    <t>app/main.py / app/trip.html</t>
+  </si>
+  <si>
+    <t>車移動の予定に「経由地（IC・JCTなど）」を複数指定できる機能を追加。/api/routeを複数地点対応のPOSTに変更し、指定した経由地を通る実ルートを地図に反映</t>
   </si>
 </sst>
 </file>
@@ -638,7 +659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62BC3060-54A5-4605-B70E-1E9C84D367F5}">
-  <dimension ref="A1:CA30"/>
+  <dimension ref="A1:CA35"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1489,6 +1510,106 @@
         <v>22259</v>
       </c>
     </row>
+    <row r="31" spans="1:79">
+      <c r="A31" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="32" spans="1:79">
+      <c r="A32" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6">
+      <c r="A35" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Log v1.6 trip deletion, button restyle, forest palette, and bug fixes in changelog
</commit_message>
<xml_diff>
--- a/tripplanner_changelog.xlsx
+++ b/tripplanner_changelog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gogle\Claude\Projects\TripPlanner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D91779FD-A234-4A6A-8AEF-4A7C9BA28FC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70AF326E-174A-4B19-8A20-919DE2040D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="465" yWindow="1650" windowWidth="23760" windowHeight="17655" xr2:uid="{86CE85FA-8EFB-405C-82A3-7763046D7446}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="79">
   <si>
     <t>バージョン</t>
   </si>
@@ -249,6 +249,33 @@
   </si>
   <si>
     <t>車移動の予定に「経由地（IC・JCTなど）」を複数指定できる機能を追加。/api/routeを複数地点対応のPOSTに変更し、指定した経由地を通る実ルートを地図に反映</t>
+  </si>
+  <si>
+    <t>v1.6</t>
+  </si>
+  <si>
+    <t>旅行削除機能を追加（タイトル横の🗑️アイコン→確認モーダルで2段階確認）</t>
+  </si>
+  <si>
+    <t>「予定を追加」「日を追加」ボタンを小さく、日を追加はタン系の色に変更</t>
+  </si>
+  <si>
+    <t>app/index.html / app/trip.html</t>
+  </si>
+  <si>
+    <t>配色をテラコッタからフォレスト（緑）に変更。選択中プランは帯スタイル、日付バッジは輪郭スタイルにして役割ごとに視覚的差をつけた</t>
+  </si>
+  <si>
+    <t>画面全体</t>
+  </si>
+  <si>
+    <t>不具合修正: 旅行作成モーダルの開始日/終了日欄の幅が不揃いだったのを均等幅に修正</t>
+  </si>
+  <si>
+    <t>旅行作成</t>
+  </si>
+  <si>
+    <t>「日を追加」で日付を選べず自動連番だった問題を修正。日付選択モーダルを追加し、追加後は日付順に並び替え</t>
   </si>
 </sst>
 </file>
@@ -659,7 +686,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62BC3060-54A5-4605-B70E-1E9C84D367F5}">
-  <dimension ref="A1:CA35"/>
+  <dimension ref="A1:CA40"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1610,6 +1637,106 @@
         <v>40</v>
       </c>
     </row>
+    <row r="36" spans="1:6">
+      <c r="A36" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6">
+      <c r="A37" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6">
+      <c r="A38" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6">
+      <c r="A39" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6">
+      <c r="A40" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Log v1.7 map removal, AI origin field, and version display in changelog
</commit_message>
<xml_diff>
--- a/tripplanner_changelog.xlsx
+++ b/tripplanner_changelog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gogle\Claude\Projects\TripPlanner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70AF326E-174A-4B19-8A20-919DE2040D85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A80150C-B250-4CAE-94F8-DFB767CC547C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="465" yWindow="1650" windowWidth="23760" windowHeight="17655" xr2:uid="{86CE85FA-8EFB-405C-82A3-7763046D7446}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="87">
   <si>
     <t>バージョン</t>
   </si>
@@ -276,6 +276,30 @@
   </si>
   <si>
     <t>「日を追加」で日付を選べず自動連番だった問題を修正。日付選択モーダルを追加し、追加後は日付順に並び替え</t>
+  </si>
+  <si>
+    <t>v1.7</t>
+  </si>
+  <si>
+    <t>2026/07/15</t>
+  </si>
+  <si>
+    <t>地図機能を一時停止（Leaflet読み込み・地図カード・renderMap呼び出し・経由地UIをコメントアウト）。軽量化のためだが、裏側のロジックは全て残しコメントを外すだけで復帰可能。場所欄は自由入力テキストに変更</t>
+  </si>
+  <si>
+    <t>旅程・地図</t>
+  </si>
+  <si>
+    <t>app/trip.html / app/main.py</t>
+  </si>
+  <si>
+    <t>AI旅程提案に「出発地（任意）」欄を追加。入力すると1日目がその出発地から始まる旅程を生成</t>
+  </si>
+  <si>
+    <t>app/trip.html / app/index.html</t>
+  </si>
+  <si>
+    <t>ヘッダーとログイン画面にバージョン番号（v1.7）を表示</t>
   </si>
 </sst>
 </file>
@@ -686,7 +710,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62BC3060-54A5-4605-B70E-1E9C84D367F5}">
-  <dimension ref="A1:CA40"/>
+  <dimension ref="A1:CA43"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1737,6 +1761,66 @@
         <v>37</v>
       </c>
     </row>
+    <row r="41" spans="1:6">
+      <c r="A41" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6">
+      <c r="A42" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6">
+      <c r="A43" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Log v1.8 budget reposition and yen display in changelog
</commit_message>
<xml_diff>
--- a/tripplanner_changelog.xlsx
+++ b/tripplanner_changelog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gogle\Claude\Projects\TripPlanner\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A80150C-B250-4CAE-94F8-DFB767CC547C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1BC45E9-4309-4BC7-AC28-E47460627040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="465" yWindow="1650" windowWidth="23760" windowHeight="17655" xr2:uid="{86CE85FA-8EFB-405C-82A3-7763046D7446}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="90">
   <si>
     <t>バージョン</t>
   </si>
@@ -300,6 +300,15 @@
   </si>
   <si>
     <t>ヘッダーとログイン画面にバージョン番号（v1.7）を表示</t>
+  </si>
+  <si>
+    <t>v1.8</t>
+  </si>
+  <si>
+    <t>予算カードをプラン名の直下（旅程カードの上）に移動</t>
+  </si>
+  <si>
+    <t>金額表示をJPYから「円」に変更し、通貨を円固定にシンプル化（予定入力の通貨欄を削除、合計は全額を単純合算）</t>
   </si>
 </sst>
 </file>
@@ -710,7 +719,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{62BC3060-54A5-4605-B70E-1E9C84D367F5}">
-  <dimension ref="A1:CA43"/>
+  <dimension ref="A1:CA45"/>
   <sheetFormatPr defaultRowHeight="18.75"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1821,6 +1830,46 @@
         <v>75</v>
       </c>
     </row>
+    <row r="44" spans="1:6">
+      <c r="A44" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>